<commit_message>
Atualizacao automatica empregados terceirizados
</commit_message>
<xml_diff>
--- a/de_para_orgao.xlsx
+++ b/de_para_orgao.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="138">
   <si>
     <t>para_orgao</t>
   </si>
@@ -449,6 +449,9 @@
   </si>
   <si>
     <t>SEDE</t>
+  </si>
+  <si>
+    <t>DMAES PONTE NOVA</t>
   </si>
 </sst>
 </file>
@@ -1258,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -2036,6 +2039,17 @@
         <v>123</v>
       </c>
     </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>137</v>
+      </c>
+      <c r="B71" t="s">
+        <v>133</v>
+      </c>
+      <c r="C71" t="s">
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1">
     <sortState ref="A2:C61">

</xml_diff>